<commit_message>
Weekly накладная: swap in the corrected template
The user sent an updated weekly-invoice-template.xlsx (different file, not
just a resend) — install that one in place of the earlier version. Column
layout changed: no more Единицы измерения column, and 'Заказы' is now
explicitly 'Номер заказа' with a literal №000-prefixed token, which
downloadWeeklyInvoiceExcel now reads off the template itself (rather than
hand-transcribing — this template's own [total_amount]-equivalent token
turned out to have a Cyrillic о baked in, invisible at a glance). fillToken
is now bracket-agnostic (matches the cell's one [..] run rather than a
literal token string) so a future template's typo'd token name can't
silently no-op a header substitution again.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/assets/templates/weekly-invoice-template.xlsx
+++ b/src/assets/templates/weekly-invoice-template.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>&lt;order&gt;</t>
   </si>
@@ -35,18 +35,9 @@
     <t>Организация: [client_company_name]</t>
   </si>
   <si>
-    <t>Дата заявки:  [date]</t>
-  </si>
-  <si>
-    <t>Единицы измерения</t>
-  </si>
-  <si>
     <t>НДС</t>
   </si>
   <si>
-    <t>[measure_short_name]</t>
-  </si>
-  <si>
     <t>[vat_sum]</t>
   </si>
   <si>
@@ -62,35 +53,38 @@
     <t>&lt;product&gt;[order_no]</t>
   </si>
   <si>
-    <t>Заказы</t>
-  </si>
-  <si>
     <t>Обшая сумма заказа</t>
   </si>
   <si>
-    <t>Итого: [total_amaunt]</t>
-  </si>
-  <si>
     <t>Дата</t>
   </si>
   <si>
     <t>[order_date]</t>
   </si>
   <si>
-    <t>[order_number]</t>
-  </si>
-  <si>
     <t>Сумма без ндс</t>
   </si>
   <si>
     <t>[sum_without_vat]</t>
+  </si>
+  <si>
+    <t>Номер заказа</t>
+  </si>
+  <si>
+    <t>Итого: [total_amоunt]</t>
+  </si>
+  <si>
+    <t>№000[order_number]</t>
+  </si>
+  <si>
+    <t>Дата:[date]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -134,6 +128,15 @@
       <color rgb="FF0C0C0C"/>
       <name val="sans-serif"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -160,7 +163,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -218,17 +221,6 @@
     </border>
     <border>
       <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right/>
       <top style="medium">
         <color indexed="64"/>
@@ -264,14 +256,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -280,10 +271,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -296,48 +289,39 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -347,20 +331,17 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -642,14 +623,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="9" max="11" width="9.140625" customWidth="1"/>
+    <col min="7" max="8" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:13">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
@@ -658,132 +639,122 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:16">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:13">
+      <c r="A2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:16" ht="15" customHeight="1">
-      <c r="A3" s="33" t="s">
+    <row r="3" spans="1:13" ht="15" customHeight="1">
+      <c r="A3" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="33"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
     </row>
-    <row r="4" spans="1:16" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A4" s="34" t="s">
+    <row r="4" spans="1:13" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A4" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="27"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+    </row>
+    <row r="5" spans="1:13" ht="15.75" thickBot="1">
+      <c r="A5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="25"/>
+      <c r="D5" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="24"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="20"/>
+      <c r="I5" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="L5" s="17"/>
+      <c r="M5" s="18"/>
     </row>
-    <row r="5" spans="1:16" ht="15.75" thickBot="1">
-      <c r="A5" s="4" t="s">
+    <row r="6" spans="1:13" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B6" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="15"/>
+      <c r="D6" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="14"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="22"/>
+      <c r="I6" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="J6" s="15"/>
+      <c r="K6" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="L6" s="14"/>
+      <c r="M6" s="15"/>
+    </row>
+    <row r="7" spans="1:13" ht="15.75" thickBot="1">
+      <c r="K7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="29"/>
-      <c r="D5" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="28"/>
-      <c r="F5" s="29"/>
-      <c r="G5" s="30" t="s">
-        <v>4</v>
-      </c>
-      <c r="H5" s="31"/>
-      <c r="I5" s="32"/>
-      <c r="J5" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="K5" s="26"/>
-      <c r="L5" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="M5" s="13"/>
-      <c r="N5" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="O5" s="23"/>
-      <c r="P5" s="24"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="10"/>
     </row>
-    <row r="6" spans="1:16" ht="15.75" thickBot="1">
-      <c r="A6" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" s="15"/>
-      <c r="F6" s="16"/>
-      <c r="G6" s="17" t="s">
-        <v>6</v>
-      </c>
-      <c r="H6" s="18"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="K6" s="19"/>
-      <c r="L6" s="20" t="s">
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="M6" s="21"/>
-      <c r="N6" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="O6" s="15"/>
-      <c r="P6" s="16"/>
-    </row>
-    <row r="7" spans="1:16" ht="15.75" thickBot="1">
-      <c r="N7" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="O7" s="10"/>
-      <c r="P7" s="11"/>
-    </row>
-    <row r="8" spans="1:16">
-      <c r="A8" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="14">
+    <mergeCell ref="A2:D2"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="G5:I5"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="N7:P7"/>
-    <mergeCell ref="L5:M5"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="K7:M7"/>
+    <mergeCell ref="I5:J5"/>
     <mergeCell ref="D6:F6"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="N6:P6"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="J5:K5"/>
-    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="K6:M6"/>
+    <mergeCell ref="K5:M5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
     <mergeCell ref="D5:F5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Weekly накладная: swap in the latest template (again)
Another revised weekly-invoice-template.xlsx — Номер заказа is back to a
single unmerged column with just [order_number] (no literal prefix this
time; the prefix-extraction code already tolerates that — it reads
whatever's actually there instead of assuming one exists). Column count
dropped from 13 to 11 (Сумма без ндс / НДС / Обшая сумма заказа are now
narrower groups).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/assets/templates/weekly-invoice-template.xlsx
+++ b/src/assets/templates/weekly-invoice-template.xlsx
@@ -74,10 +74,10 @@
     <t>Итого: [total_amоunt]</t>
   </si>
   <si>
-    <t>№000[order_number]</t>
-  </si>
-  <si>
     <t>Дата:[date]</t>
+  </si>
+  <si>
+    <t>[order_number]</t>
   </si>
 </sst>
 </file>
@@ -256,27 +256,48 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -292,15 +313,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -321,27 +336,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -623,114 +617,102 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="7" max="8" width="9.140625" customWidth="1"/>
+    <col min="5" max="6" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:11">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:13">
-      <c r="A2" s="29" t="s">
+    <row r="2" spans="1:11">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
     </row>
-    <row r="3" spans="1:13" ht="15" customHeight="1">
-      <c r="A3" s="26" t="s">
+    <row r="3" spans="1:11" ht="15" customHeight="1">
+      <c r="A3" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:13" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A4" s="27" t="s">
+    <row r="4" spans="1:11" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A4" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="14"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="12"/>
+      <c r="D5" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="25"/>
+      <c r="G5" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="H5" s="19"/>
+      <c r="I5" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="J5" s="22"/>
+      <c r="K5" s="23"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="10"/>
+      <c r="D6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
+      <c r="E6" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="27"/>
+      <c r="G6" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="H6" s="10"/>
+      <c r="I6" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="J6" s="20"/>
+      <c r="K6" s="10"/>
     </row>
-    <row r="5" spans="1:13" ht="15.75" thickBot="1">
-      <c r="A5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="24"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="H5" s="20"/>
-      <c r="I5" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="J5" s="12"/>
-      <c r="K5" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="L5" s="17"/>
-      <c r="M5" s="18"/>
+    <row r="7" spans="1:11" ht="15.75" thickBot="1">
+      <c r="I7" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="J7" s="16"/>
+      <c r="K7" s="17"/>
     </row>
-    <row r="6" spans="1:13" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A6" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="14"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" s="22"/>
-      <c r="I6" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="J6" s="15"/>
-      <c r="K6" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="L6" s="14"/>
-      <c r="M6" s="15"/>
-    </row>
-    <row r="7" spans="1:13" ht="15.75" thickBot="1">
-      <c r="K7" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="L7" s="9"/>
-      <c r="M7" s="10"/>
-    </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:11">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -738,21 +720,19 @@
       <c r="C8" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="12">
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="I6:K6"/>
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E6:F6"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="K7:M7"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="K6:M6"/>
-    <mergeCell ref="K5:M5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="D5:F5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>